<commit_message>
Adjust Excel and PDF exports by removing status and resizing columns
Remove the "Durum" column from PDF and Excel exports, adjust column widths, and update the Excel sheet layout.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 5b104115-5f33-4fe7-8253-bfe4d0792bb1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 57092d96-2844-495a-9251-137a9d32bc5b
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e6d0ee3d-1217-42e6-be43-c7e0ae7e577a/5b104115-5f33-4fe7-8253-bfe4d0792bb1/EUTEyE8
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/sample-output/ornek-ekstre.xlsx
+++ b/artifacts/api-server/sample-output/ornek-ekstre.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="40">
   <si>
     <t>CARİ HESAP EKSTRESİ</t>
   </si>
@@ -76,9 +76,6 @@
     <t>Bakiye</t>
   </si>
   <si>
-    <t>Durum</t>
-  </si>
-  <si>
     <t>01.06.2026</t>
   </si>
   <si>
@@ -91,9 +88,6 @@
     <t>15.06.2026</t>
   </si>
   <si>
-    <t>Kısmi</t>
-  </si>
-  <si>
     <t>10.06.2026</t>
   </si>
   <si>
@@ -106,18 +100,12 @@
     <t>20.06.2026</t>
   </si>
   <si>
-    <t>Ödendi</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
     <t>Tahsilat — Haziran kısmi</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>Tahsilat — MAG000002 kapanış</t>
   </si>
   <si>
@@ -131,9 +119,6 @@
   </si>
   <si>
     <t>15.07.2026</t>
-  </si>
-  <si>
-    <t>Açık</t>
   </si>
   <si>
     <t>MAG000004</t>
@@ -578,19 +563,18 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="38" customWidth="1"/>
+    <col min="3" max="3" width="58" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -600,73 +584,72 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
     </row>
     <row r="2" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" ht="18" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="4">
+      <c r="G4" s="4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B5" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="F5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="4">
+      <c r="G5" s="4">
         <v>5800</v>
       </c>
     </row>
-    <row r="6" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B6" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="F6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="4">
+      <c r="G6" s="4">
         <v>2850</v>
       </c>
     </row>
-    <row r="7" ht="16" customHeight="1" spans="7:8" x14ac:dyDescent="0.25">
-      <c r="G7" s="2" t="s">
+    <row r="7" ht="16" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="5">
+      <c r="G7" s="5">
         <v>2950</v>
       </c>
     </row>
     <row r="8" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="9" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>14</v>
       </c>
@@ -688,22 +671,19 @@
       <c r="G9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="6" t="s">
+    </row>
+    <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+      <c r="B10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="E10" s="8">
         <v>2500</v>
@@ -712,22 +692,19 @@
       <c r="G10" s="9">
         <v>2500</v>
       </c>
-      <c r="H10" s="7" t="s">
+    </row>
+    <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="11" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="C11" t="s">
         <v>27</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
         <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" t="s">
-        <v>30</v>
       </c>
       <c r="E11" s="10">
         <v>350</v>
@@ -735,22 +712,19 @@
       <c r="G11" s="11">
         <v>2850</v>
       </c>
-      <c r="H11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E12" s="7"/>
       <c r="F12" s="8">
@@ -759,22 +733,19 @@
       <c r="G12" s="9">
         <v>850</v>
       </c>
-      <c r="H12" s="7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F13" s="10">
         <v>350</v>
@@ -782,22 +753,19 @@
       <c r="G13" s="11">
         <v>500</v>
       </c>
-      <c r="H13" t="s">
+    </row>
+    <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="14" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>38</v>
-      </c>
       <c r="D14" s="7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E14" s="8">
         <v>2500</v>
@@ -806,22 +774,19 @@
       <c r="G14" s="9">
         <v>3000</v>
       </c>
-      <c r="H14" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" t="s">
         <v>36</v>
       </c>
-      <c r="B15" t="s">
-        <v>41</v>
-      </c>
       <c r="C15" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D15" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E15" s="10">
         <v>450</v>
@@ -829,22 +794,19 @@
       <c r="G15" s="11">
         <v>3450</v>
       </c>
-      <c r="H15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E16" s="7"/>
       <c r="F16" s="8">
@@ -853,14 +815,11 @@
       <c r="G16" s="9">
         <v>2950</v>
       </c>
-      <c r="H16" s="7" t="s">
-        <v>34</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="F3:G3"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>

<commit_message>
Improve report layout by adjusting column widths
Update PDF and Excel report column widths to improve readability and accommodate longer descriptions.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 5b104115-5f33-4fe7-8253-bfe4d0792bb1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 1cb77b50-bc66-4acf-9dd5-bc866d0c7b50
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e6d0ee3d-1217-42e6-be43-c7e0ae7e577a/5b104115-5f33-4fe7-8253-bfe4d0792bb1/EUTEyE8
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/sample-output/ornek-ekstre.xlsx
+++ b/artifacts/api-server/sample-output/ornek-ekstre.xlsx
@@ -94,7 +94,7 @@
     <t>MAG000002</t>
   </si>
   <si>
-    <t>Ek Veri Paketi — MV SEBA</t>
+    <t>Ek Veri Paketi — MV SEBA (Haziran ayı ek kullanım)</t>
   </si>
   <si>
     <t>20.06.2026</t>
@@ -103,10 +103,10 @@
     <t/>
   </si>
   <si>
-    <t>Tahsilat — Haziran kısmi</t>
-  </si>
-  <si>
-    <t>Tahsilat — MAG000002 kapanış</t>
+    <t>Tahsilat — Haziran kısmi ödeme / Banka Havalesi</t>
+  </si>
+  <si>
+    <t>Tahsilat — MAG000002 kapanış ödemesi</t>
   </si>
   <si>
     <t>01.07.2026</t>
@@ -124,13 +124,13 @@
     <t>MAG000004</t>
   </si>
   <si>
-    <t>Donanım Kiralama — Antena Ünitesi</t>
+    <t>Donanım Kiralama — Uydu Antena Ünitesi (Temmuz 2026)</t>
   </si>
   <si>
     <t>06.07.2026</t>
   </si>
   <si>
-    <t>Tahsilat — Haziran bakiye kapanış</t>
+    <t>Tahsilat — Haziran bakiye kapanış ödemesi</t>
   </si>
 </sst>
 </file>
@@ -568,7 +568,7 @@
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="58" customWidth="1"/>
+    <col min="3" max="3" width="68" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="6" width="14" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>

</xml_diff>

<commit_message>
Move summary section to bottom of reports
Reposition the summary section in PDF and Excel exports from the header to below the data rows, and fix a column count bug in Excel.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 5b104115-5f33-4fe7-8253-bfe4d0792bb1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e74bbe38-f880-4078-8826-01161af26099
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e6d0ee3d-1217-42e6-be43-c7e0ae7e577a/5b104115-5f33-4fe7-8253-bfe4d0792bb1/EUTEyE8
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/artifacts/api-server/sample-output/ornek-ekstre.xlsx
+++ b/artifacts/api-server/sample-output/ornek-ekstre.xlsx
@@ -22,115 +22,115 @@
     <t>Dragos Shipping Limited</t>
   </si>
   <si>
+    <t>Ekstre Tarih Aralığı</t>
+  </si>
+  <si>
+    <t>01.06.2026 / 06.07.2026</t>
+  </si>
+  <si>
+    <t>Para Birimi</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>Hazırlayan</t>
+  </si>
+  <si>
+    <t>ADE GlobaSpace LIMITED</t>
+  </si>
+  <si>
+    <t>Tarih</t>
+  </si>
+  <si>
+    <t>Belge No</t>
+  </si>
+  <si>
+    <t>Açıklama</t>
+  </si>
+  <si>
+    <t>Vade Tarihi</t>
+  </si>
+  <si>
+    <t>Borç</t>
+  </si>
+  <si>
+    <t>Alacak</t>
+  </si>
+  <si>
+    <t>Bakiye</t>
+  </si>
+  <si>
+    <t>01.06.2026</t>
+  </si>
+  <si>
+    <t>MAG000001</t>
+  </si>
+  <si>
+    <t>Starlink Hizmet Bedeli Haziran 2026</t>
+  </si>
+  <si>
+    <t>15.06.2026</t>
+  </si>
+  <si>
+    <t>10.06.2026</t>
+  </si>
+  <si>
+    <t>MAG000002</t>
+  </si>
+  <si>
+    <t>Ek Veri Paketi — MV SEBA (Haziran ayı ek kullanım)</t>
+  </si>
+  <si>
+    <t>20.06.2026</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Tahsilat — Haziran kısmi ödeme / Banka Havalesi</t>
+  </si>
+  <si>
+    <t>Tahsilat — MAG000002 kapanış ödemesi</t>
+  </si>
+  <si>
+    <t>01.07.2026</t>
+  </si>
+  <si>
+    <t>MAG000003</t>
+  </si>
+  <si>
+    <t>Starlink Hizmet Bedeli Temmuz 2026</t>
+  </si>
+  <si>
+    <t>15.07.2026</t>
+  </si>
+  <si>
+    <t>MAG000004</t>
+  </si>
+  <si>
+    <t>Donanım Kiralama — Uydu Antena Ünitesi (Temmuz 2026)</t>
+  </si>
+  <si>
+    <t>06.07.2026</t>
+  </si>
+  <si>
+    <t>Tahsilat — Haziran bakiye kapanış ödemesi</t>
+  </si>
+  <si>
     <t>ÖZET</t>
   </si>
   <si>
-    <t>Ekstre Tarih Aralığı</t>
-  </si>
-  <si>
-    <t>01.06.2026 / 06.07.2026</t>
-  </si>
-  <si>
     <t>Açılış Bakiyesi</t>
   </si>
   <si>
-    <t>Para Birimi</t>
-  </si>
-  <si>
-    <t>USD</t>
-  </si>
-  <si>
     <t>Toplam Borç</t>
   </si>
   <si>
-    <t>Hazırlayan</t>
-  </si>
-  <si>
-    <t>ADE GlobaSpace LIMITED</t>
-  </si>
-  <si>
     <t>Toplam Alacak</t>
   </si>
   <si>
     <t>Kapanış Bakiyesi</t>
-  </si>
-  <si>
-    <t>Tarih</t>
-  </si>
-  <si>
-    <t>Belge No</t>
-  </si>
-  <si>
-    <t>Açıklama</t>
-  </si>
-  <si>
-    <t>Vade Tarihi</t>
-  </si>
-  <si>
-    <t>Borç</t>
-  </si>
-  <si>
-    <t>Alacak</t>
-  </si>
-  <si>
-    <t>Bakiye</t>
-  </si>
-  <si>
-    <t>01.06.2026</t>
-  </si>
-  <si>
-    <t>MAG000001</t>
-  </si>
-  <si>
-    <t>Starlink Hizmet Bedeli Haziran 2026</t>
-  </si>
-  <si>
-    <t>15.06.2026</t>
-  </si>
-  <si>
-    <t>10.06.2026</t>
-  </si>
-  <si>
-    <t>MAG000002</t>
-  </si>
-  <si>
-    <t>Ek Veri Paketi — MV SEBA (Haziran ayı ek kullanım)</t>
-  </si>
-  <si>
-    <t>20.06.2026</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Tahsilat — Haziran kısmi ödeme / Banka Havalesi</t>
-  </si>
-  <si>
-    <t>Tahsilat — MAG000002 kapanış ödemesi</t>
-  </si>
-  <si>
-    <t>01.07.2026</t>
-  </si>
-  <si>
-    <t>MAG000003</t>
-  </si>
-  <si>
-    <t>Starlink Hizmet Bedeli Temmuz 2026</t>
-  </si>
-  <si>
-    <t>15.07.2026</t>
-  </si>
-  <si>
-    <t>MAG000004</t>
-  </si>
-  <si>
-    <t>Donanım Kiralama — Uydu Antena Ünitesi (Temmuz 2026)</t>
-  </si>
-  <si>
-    <t>06.07.2026</t>
-  </si>
-  <si>
-    <t>Tahsilat — Haziran bakiye kapanış ödemesi</t>
   </si>
 </sst>
 </file>
@@ -156,17 +156,13 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b/>
-      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <b/>
       <color rgb="FFCA8A04"/>
     </font>
+    <font/>
   </fonts>
   <fills count="4">
     <fill>
@@ -207,20 +203,18 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,7 +557,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="F1:G22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -586,240 +580,250 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="3" ht="18" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" ht="18" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="3" t="s">
+    </row>
+    <row r="4" ht="16" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="3"/>
-    </row>
-    <row r="4" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+    </row>
+    <row r="5" ht="16" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+    </row>
+    <row r="6" ht="16" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="4">
-        <v>5800</v>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="4">
-        <v>2850</v>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
-      <c r="F7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="5">
-        <v>2950</v>
-      </c>
-    </row>
+    </row>
+    <row r="7" ht="16" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="8" ht="10" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="9" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="G9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="6" t="s">
+    </row>
+    <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="C10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="D10" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="8">
+      <c r="E10" s="5">
         <v>2500</v>
       </c>
-      <c r="F10" s="7"/>
-      <c r="G10" s="9">
+      <c r="F10" s="4"/>
+      <c r="G10" s="6">
         <v>2500</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="7">
+        <v>350</v>
+      </c>
+      <c r="G11" s="8">
+        <v>2850</v>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" s="10">
-        <v>350</v>
-      </c>
-      <c r="G11" s="11">
-        <v>2850</v>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="D12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="8">
+      <c r="E12" s="4"/>
+      <c r="F12" s="5">
         <v>2000</v>
       </c>
-      <c r="G12" s="9">
+      <c r="G12" s="6">
         <v>850</v>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" t="s">
+        <v>26</v>
+      </c>
+      <c r="D13" t="s">
+        <v>24</v>
+      </c>
+      <c r="F13" s="7">
+        <v>350</v>
+      </c>
+      <c r="G13" s="8">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C14" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C13" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" t="s">
-        <v>29</v>
-      </c>
-      <c r="F13" s="10">
-        <v>350</v>
-      </c>
-      <c r="G13" s="11">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="8">
+      <c r="D14" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" s="5">
         <v>2500</v>
       </c>
-      <c r="F14" s="7"/>
-      <c r="G14" s="9">
+      <c r="F14" s="4"/>
+      <c r="G14" s="6">
         <v>3000</v>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" t="s">
         <v>32</v>
       </c>
-      <c r="B15" t="s">
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" s="7">
+        <v>450</v>
+      </c>
+      <c r="G15" s="8">
+        <v>3450</v>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="4"/>
+      <c r="F16" s="5">
+        <v>500</v>
+      </c>
+      <c r="G16" s="6">
+        <v>2950</v>
+      </c>
+    </row>
+    <row r="17" ht="8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" ht="18" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F18" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G18" s="3"/>
+    </row>
+    <row r="19" ht="16" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F19" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C15" t="s">
+      <c r="G19" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F20" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D15" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="10">
-        <v>450</v>
-      </c>
-      <c r="G15" s="11">
-        <v>3450</v>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
+      <c r="G20" s="10">
+        <v>5800</v>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F21" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C16" s="7" t="s">
+      <c r="G21" s="10">
+        <v>2850</v>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1" spans="6:7" x14ac:dyDescent="0.25">
+      <c r="F22" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="8">
-        <v>500</v>
-      </c>
-      <c r="G16" s="9">
+      <c r="G22" s="11">
         <v>2950</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F18:G18"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>

</xml_diff>